<commit_message>
R2 requirements discussion planning docs
</commit_message>
<xml_diff>
--- a/KT_Session_Question_Review/SHRSS_Adobe_KT_Session_Questions_Flagged.xlsx
+++ b/KT_Session_Question_Review/SHRSS_Adobe_KT_Session_Questions_Flagged.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lambert/Documents/Projects/SHRSS/SHRSS_Knowledge_Transfer/KT_Session_Question_Review/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A12FA171-505F-A24E-874F-6FF9D428FDA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65329BBE-02CD-5747-8F83-0B31F404320C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="760" windowWidth="30900" windowHeight="21520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1100" yWindow="760" windowWidth="30900" windowHeight="21520" firstSheet="5" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All_Questions" sheetId="1" r:id="rId1"/>
@@ -27672,7 +27672,7 @@
     <col min="1" max="1" width="29.85546875" customWidth="1"/>
     <col min="2" max="2" width="17.42578125" customWidth="1"/>
     <col min="3" max="3" width="11.85546875" customWidth="1"/>
-    <col min="4" max="4" width="24.7109375" customWidth="1"/>
+    <col min="4" max="4" width="72.7109375" customWidth="1"/>
     <col min="5" max="5" width="26.85546875" customWidth="1"/>
     <col min="6" max="6" width="23.28515625" customWidth="1"/>
   </cols>

</xml_diff>